<commit_message>
Revert "Nothing lists a CE mark"
This reverts commit 6eee9f450bf15b399f65b6cf9dd3c933ef21279e.
</commit_message>
<xml_diff>
--- a/tools/audit/GP1-MUR lighting certification review.xlsx
+++ b/tools/audit/GP1-MUR lighting certification review.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>UL / NRTL listing</t>
+          <t>UL / NRTL</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>CE, SELV, IP20, NFC, DALI-2</t>
+          <t>CE, DALI-2</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Badge row under the product photo, page 2 (logos)</t>
+          <t>Mark strip, page 2 (logos)</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>UK driver. CE only - which is EcoPac's own declaration, not a third-party listing. No NRTL mark, though the input is 100-277 VAC and so covers US voltages.</t>
+          <t>UK driver. CE and DALI-2 only; no NRTL mark on the sheet.</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
@@ -782,12 +782,12 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>CE, SELV, IP20, NFC, DALI-2</t>
+          <t>CE, DALI-2</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Badge row under the product photo, page 2 (logos)</t>
+          <t>Mark strip, page 2 (logos)</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -795,11 +795,7 @@
           <t>Read by eye</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>CE is EcoPac's own declaration, not a third-party listing.</t>
-        </is>
-      </c>
+      <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -968,12 +964,12 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>CE, SELV, IP20, NFC, DALI-2</t>
+          <t>CE, DALI-2</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Badge row under the product photo, page 2 (logos)</t>
+          <t>Mark strip, page 2 (logos)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -981,11 +977,7 @@
           <t>Read by eye</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>CE is EcoPac's own declaration, not a third-party listing.</t>
-        </is>
-      </c>
+      <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1030,12 +1022,12 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>CE, SELV, IP20, NFC, DALI-2</t>
+          <t>CE, DALI-2</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Badge row under the product photo, page 2 (logos)</t>
+          <t>Mark strip, page 2 (logos)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1043,11 +1035,7 @@
           <t>Read by eye</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>CE is EcoPac's own declaration, not a third-party listing.</t>
-        </is>
-      </c>
+      <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1216,12 +1204,12 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>CE, SELV, IP20, NFC, DALI-2</t>
+          <t>CE, DALI-2</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Badge row under the product photo, page 2 (logos)</t>
+          <t>Mark strip, page 2 (logos)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1229,11 +1217,7 @@
           <t>Read by eye</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>CE is EcoPac's own declaration, not a third-party listing.</t>
-        </is>
-      </c>
+      <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1402,12 +1386,12 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>CE, SELV, IP20, NFC, DALI-2</t>
+          <t>CE, DALI-2</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Badge row under the product photo, page 2 (logos)</t>
+          <t>Mark strip, page 2 (logos)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1415,11 +1399,7 @@
           <t>Read by eye</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>CE is EcoPac's own declaration, not a third-party listing. SEPARATELY: this driver is IP20 and its own sheet says "IP20 design for indoor installation", while it serves LUM6 at IP65 outdoors. Remote-mounting a driver indoors is normal, but confirm where this one actually sits.</t>
-        </is>
-      </c>
+      <c r="K17" s="5" t="inlineStr"/>
       <c r="L17" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1770,12 +1750,12 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>CE, SELV, IP20, NFC, DALI-2</t>
+          <t>CE, DALI-2</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Badge row under the product photo, page 2 (logos)</t>
+          <t>Mark strip, page 2 (logos)</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -1783,11 +1763,7 @@
           <t>Read by eye</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>CE is EcoPac's own declaration, not a third-party listing. SEPARATELY: this driver is IP20 and its own sheet says "IP20 design for indoor installation", while it serves LUM9 at IP67 outdoors. Remote-mounting a driver indoors is normal, but confirm where this one actually sits.</t>
-        </is>
-      </c>
+      <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -5274,7 +5250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5301,113 +5277,101 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>A SIGNATURE, NOT A TEST. The manufacturer declares the product meets the applicable EU directives and signs a Declaration of Conformity. No third party tests it, there is no file number and there is no register to look it up in. Yes = a CE or UKCA mark appears on the sheet. Not stated = it does not, which is not the same as 'not CE marked'. Nothing 'lists' a CE mark.</t>
+          <t>Yes = a CE mark or an EU/UKCA declaration appears on the sheet. Not stated = it does not, which is not the same as 'not CE marked'.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>UL / NRTL listing</t>
+          <t>UL / NRTL</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>A TEST. A Nationally Recognized Testing Laboratory tested the product, keeps a file on it and audits the factory - UL, ETL (Intertek) or CSA - and it comes with a file number you can look up. Only a LISTING counts here. cURus = Recognized Component, valid only inside other listed equipment, not as a standalone device.</t>
+          <t>A Nationally Recognized Testing Laboratory listing: UL, ETL (Intertek) or CSA. Only a LISTING counts here. cURus = Recognized Component, which is valid only inside other listed equipment.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Why they are separate columns</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Neither substitutes for the other, and a CE mark is not a weaker grade of a UL listing - it is a different kind of claim, made by a different party.</t>
+          <t>Both a CE/EU mark and an NRTL listing are stated.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Amber</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Both a CE/EU mark and an NRTL listing are stated.</t>
+          <t>One of the two is stated.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Amber</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>One of the two is stated.</t>
+          <t>Neither is stated, or a listing is marked pending.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Grey</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Neither is stated, or a listing is marked pending.</t>
+          <t>Not an electrical product - a bare extrusion carries no listing.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>Grey</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Not an electrical product - a bare extrusion carries no listing.</t>
-        </is>
-      </c>
+      <c r="A8" s="14" t="inlineStr"/>
+      <c r="B8" s="15" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr"/>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Two traps this review was built to avoid</t>
+        </is>
+      </c>
       <c r="B9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Two traps this review was built to avoid</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr"/>
+          <t>A standard is not a listing</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>"Standards compliance: CSA C22.2 no. 223" and "Safety standards ... UL8750 UL1310" say what a product was designed to. Anyone may write that. A listing is a body saying it tested the thing, and it comes with a mark and usually a file number.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>A standard is not a listing</t>
+          <t>The marks are pictures</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>"Standards compliance: CSA C22.2 no. 223" and "Safety standards ... UL8750 UL1310" say what a product was designed to. Anyone may write that. A listing is a body saying it tested the thing, and it comes with a mark and usually a file number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>The marks are pictures</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Most of these sheets carry their marks as logos, so searching the text finds nothing on a sheet that plainly shows CE and UL. Rows marked 'Read by eye' were checked on the rendered page.</t>
         </is>

</xml_diff>